<commit_message>
Update CFC Fantasy League 2026.xlsx
</commit_message>
<xml_diff>
--- a/CFC Fantasy League 2026.xlsx
+++ b/CFC Fantasy League 2026.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,52 +490,60 @@
           <t>GT vs PBKS</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Emerging Player</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Night Watchmen</t>
+          <t>Gujju Gang</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1634</v>
+        <v>2354</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>268</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>180</v>
+        <v>119</v>
       </c>
       <c r="I2" t="n">
-        <v>278</v>
+        <v>65</v>
       </c>
       <c r="J2" t="n">
-        <v>421</v>
+        <v>242</v>
       </c>
       <c r="K2" t="n">
-        <v>337</v>
+        <v>628</v>
+      </c>
+      <c r="L2" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Nasty Knights</t>
+          <t>Tormented Titans</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1537</v>
+        <v>1880</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -544,35 +552,38 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="F3" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>770</v>
+        <v>62</v>
       </c>
       <c r="H3" t="n">
-        <v>189</v>
+        <v>272</v>
       </c>
       <c r="I3" t="n">
-        <v>15</v>
+        <v>350</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="K3" t="n">
-        <v>413</v>
+        <v>193</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Disruptors</t>
+          <t>Nasty Knights</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1489</v>
+        <v>1537</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -587,29 +598,32 @@
         <v>150</v>
       </c>
       <c r="G4" t="n">
-        <v>280</v>
+        <v>770</v>
       </c>
       <c r="H4" t="n">
-        <v>159</v>
+        <v>189</v>
       </c>
       <c r="I4" t="n">
-        <v>536</v>
+        <v>15</v>
       </c>
       <c r="J4" t="n">
-        <v>192</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>172</v>
+        <v>413</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>VS Stalwarts</t>
+          <t>Night Watchmen</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1332</v>
+        <v>1484</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -624,29 +638,32 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>348</v>
+        <v>268</v>
       </c>
       <c r="H5" t="n">
-        <v>107</v>
+        <v>180</v>
       </c>
       <c r="I5" t="n">
-        <v>157</v>
+        <v>278</v>
       </c>
       <c r="J5" t="n">
-        <v>627</v>
+        <v>421</v>
       </c>
       <c r="K5" t="n">
-        <v>93</v>
+        <v>337</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Tormented Titans</t>
+          <t>Disruptors</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1280</v>
+        <v>1339</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -658,32 +675,35 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>62</v>
+        <v>280</v>
       </c>
       <c r="H6" t="n">
-        <v>272</v>
+        <v>159</v>
       </c>
       <c r="I6" t="n">
-        <v>350</v>
+        <v>536</v>
       </c>
       <c r="J6" t="n">
-        <v>253</v>
+        <v>192</v>
       </c>
       <c r="K6" t="n">
-        <v>193</v>
+        <v>172</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Gujju Gang</t>
+          <t>VS Stalwarts</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1054</v>
+        <v>1332</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -698,19 +718,22 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>348</v>
       </c>
       <c r="H7" t="n">
-        <v>119</v>
+        <v>107</v>
       </c>
       <c r="I7" t="n">
-        <v>65</v>
+        <v>157</v>
       </c>
       <c r="J7" t="n">
-        <v>242</v>
+        <v>627</v>
       </c>
       <c r="K7" t="n">
-        <v>628</v>
+        <v>93</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -720,7 +743,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>908</v>
+        <v>758</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -732,7 +755,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="G8" t="n">
         <v>39</v>
@@ -748,6 +771,9 @@
       </c>
       <c r="K8" t="n">
         <v>15</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -785,6 +811,9 @@
       </c>
       <c r="K9" t="n">
         <v>112</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1802,11 +1831,7 @@
       <c r="B2" t="n">
         <v>192</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>6</v>
       </c>
@@ -2405,11 +2430,7 @@
       <c r="B3" t="n">
         <v>0</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
@@ -3008,11 +3029,7 @@
       <c r="B4" t="n">
         <v>421</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
@@ -3611,11 +3628,7 @@
       <c r="B5" t="n">
         <v>300</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
@@ -4214,11 +4227,7 @@
       <c r="B6" t="n">
         <v>242</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
@@ -4817,11 +4826,7 @@
       <c r="B7" t="n">
         <v>253</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
@@ -5420,11 +5425,7 @@
       <c r="B8" t="n">
         <v>627</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
@@ -6023,11 +6024,7 @@
       <c r="B9" t="n">
         <v>0</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
@@ -10589,11 +10586,7 @@
       <c r="B2" t="n">
         <v>172</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>0</v>
       </c>
@@ -11192,11 +11185,7 @@
       <c r="B3" t="n">
         <v>413</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
@@ -11795,11 +11784,7 @@
       <c r="B4" t="n">
         <v>337</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
@@ -12398,11 +12383,7 @@
       <c r="B5" t="n">
         <v>15</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
@@ -13001,11 +12982,7 @@
       <c r="B6" t="n">
         <v>628</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
@@ -13604,11 +13581,7 @@
       <c r="B7" t="n">
         <v>193</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
@@ -14207,11 +14180,7 @@
       <c r="B8" t="n">
         <v>93</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
@@ -14810,11 +14779,7 @@
       <c r="B9" t="n">
         <v>112</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
@@ -15415,7 +15380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J116"/>
+  <dimension ref="A1:K116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15464,18 +15429,23 @@
           <t>GT vs PBKS</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Emerging Player</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Noor Ahmad</t>
+          <t>Sai Sudharsan</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>269</v>
+        <v>977</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -15490,23 +15460,26 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>269</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>177</v>
+      </c>
+      <c r="K2" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Ishan Kishan</t>
+          <t>Suryakumar Yadav</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>251</v>
+        <v>801</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -15515,38 +15488,41 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>251</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Shreyas Iyer</t>
+          <t>Prasidh Krishna</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>229</v>
+        <v>492</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -15564,17 +15540,20 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>229</v>
+        <v>-8</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Krunal Pandya</t>
+          <t>Noor Ahmad</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>216</v>
+        <v>269</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -15586,29 +15565,32 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>216</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>269</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Nicholas Pooran</t>
+          <t>Ishan Kishan</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>193</v>
+        <v>251</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>
@@ -15623,26 +15605,29 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>251</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>193</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Khaleel Ahmed</t>
+          <t>Shreyas Iyer</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>190</v>
+        <v>229</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -15660,23 +15645,26 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>190</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
+        <v>229</v>
+      </c>
+      <c r="K7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Ashutosh Sharma</t>
+          <t>Krunal Pandya</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>186</v>
+        <v>216</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -15688,7 +15676,7 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>216</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -15697,20 +15685,23 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>186</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Mitchell Starc</t>
+          <t>Nicholas Pooran</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
@@ -15731,20 +15722,23 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Sai Kishore</t>
+          <t>Khaleel Ahmed</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
@@ -15762,23 +15756,26 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>190</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>184</v>
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Sai Sudharsan</t>
+          <t>Ashutosh Sharma</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
@@ -15799,20 +15796,23 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>186</v>
       </c>
       <c r="J11" t="n">
-        <v>177</v>
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Vignesh Puthur</t>
+          <t>Mitchell Starc</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
@@ -15830,23 +15830,26 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Mitchell Marsh</t>
+          <t>Sai Kishore</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
@@ -15867,20 +15870,23 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>167</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
+        <v>184</v>
+      </c>
+      <c r="K13" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Dhruv Jurel</t>
+          <t>Vignesh Puthur</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C14" t="n">
         <v>0</v>
@@ -15895,26 +15901,29 @@
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>163</v>
+        <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Travis Head</t>
+          <t>Mitchell Marsh</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="C15" t="n">
         <v>0</v>
@@ -15929,26 +15938,29 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>159</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>167</v>
       </c>
       <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Sanju Samson</t>
+          <t>Dhruv Jurel</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>
@@ -15963,7 +15975,7 @@
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -15972,17 +15984,20 @@
         <v>0</v>
       </c>
       <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Sunil Narine</t>
+          <t>Travis Head</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="C17" t="n">
         <v>0</v>
@@ -15994,10 +16009,10 @@
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>153</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -16006,17 +16021,20 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Ruturaj Gaikwad</t>
+          <t>Sanju Samson</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="C18" t="n">
         <v>0</v>
@@ -16031,26 +16049,29 @@
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="H18" t="n">
-        <v>149</v>
+        <v>0</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Kuldeep Yadav</t>
+          <t>Sunil Narine</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="C19" t="n">
         <v>0</v>
@@ -16062,7 +16083,7 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>0</v>
+        <v>153</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -16071,20 +16092,23 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>147</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Phil Salt</t>
+          <t>Ruturaj Gaikwad</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C20" t="n">
         <v>0</v>
@@ -16096,29 +16120,32 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="G20" t="n">
         <v>0</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
       <c r="J20" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Ajinkya Rahane</t>
+          <t>Kuldeep Yadav</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
@@ -16130,7 +16157,7 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -16139,20 +16166,23 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>147</v>
       </c>
       <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>Josh Hazlewood</t>
+          <t>Phil Salt</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
@@ -16164,7 +16194,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
@@ -16176,17 +16206,20 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
-          <t>Tushar Deshpande</t>
+          <t>Ajinkya Rahane</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="C23" t="n">
         <v>0</v>
@@ -16198,10 +16231,10 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="G23" t="n">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -16210,17 +16243,20 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
-          <t>Deepak Chahar</t>
+          <t>Josh Hazlewood</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
@@ -16232,29 +16268,32 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>142</v>
       </c>
       <c r="G24" t="n">
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>133</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
-          <t>Arshdeep Singh</t>
+          <t>Tushar Deshpande</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C25" t="n">
         <v>0</v>
@@ -16269,7 +16308,7 @@
         <v>0</v>
       </c>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>136</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -16278,17 +16317,20 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>132</v>
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
-          <t>Virat Kohli</t>
+          <t>Deepak Chahar</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C26" t="n">
         <v>0</v>
@@ -16300,29 +16342,32 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>131</v>
+        <v>0</v>
       </c>
       <c r="G26" t="n">
         <v>0</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>133</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>Manimaran Siddharth</t>
+          <t>Arshdeep Singh</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C27" t="n">
         <v>0</v>
@@ -16343,20 +16388,23 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>128</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
+        <v>132</v>
+      </c>
+      <c r="K27" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
-          <t>Rachin Ravindra</t>
+          <t>Virat Kohli</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C28" t="n">
         <v>0</v>
@@ -16368,29 +16416,32 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="G28" t="n">
         <v>0</v>
       </c>
       <c r="H28" t="n">
-        <v>126</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
-          <t>Digvesh Singh Rathi</t>
+          <t>Manimaran Siddharth</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C29" t="n">
         <v>0</v>
@@ -16411,20 +16462,23 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
-          <t>Jos Buttler</t>
+          <t>Rachin Ravindra</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
@@ -16442,23 +16496,26 @@
         <v>0</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>126</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>123</v>
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
-          <t>Harshal Patel</t>
+          <t>Digvesh Singh Rathi</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
@@ -16473,26 +16530,29 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
-          <t>Priyansh Arya</t>
+          <t>Jos Buttler</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C32" t="n">
         <v>0</v>
@@ -16516,17 +16576,20 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>117</v>
+        <v>123</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
-          <t>Axar Patel</t>
+          <t>Harshal Patel</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C33" t="n">
         <v>0</v>
@@ -16541,26 +16604,29 @@
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>119</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>115</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
-          <t>Shashank Singh</t>
+          <t>Priyansh Arya</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C34" t="n">
         <v>0</v>
@@ -16584,17 +16650,20 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>112</v>
+        <v>117</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>Vipraj Nigam</t>
+          <t>Axar Patel</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C35" t="n">
         <v>0</v>
@@ -16615,20 +16684,23 @@
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="inlineStr">
         <is>
-          <t>Abhishek Sharma</t>
+          <t>Shashank Singh</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C36" t="n">
         <v>0</v>
@@ -16643,7 +16715,7 @@
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -16652,17 +16724,20 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
+        <v>112</v>
+      </c>
+      <c r="K36" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
-          <t>Shimron Hetmyer</t>
+          <t>Vipraj Nigam</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C37" t="n">
         <v>0</v>
@@ -16677,26 +16752,29 @@
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
-          <t>Will Jacks</t>
+          <t>Abhishek Sharma</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="C38" t="n">
         <v>0</v>
@@ -16711,26 +16789,29 @@
         <v>0</v>
       </c>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="H38" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>Heinrich Klaasen</t>
+          <t>Shimron Hetmyer</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="C39" t="n">
         <v>0</v>
@@ -16745,7 +16826,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -16754,17 +16835,20 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>Tristan Stubbs</t>
+          <t>Will Jacks</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
@@ -16782,23 +16866,26 @@
         <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="I40" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
-          <t>Sherfane Rutherford</t>
+          <t>Heinrich Klaasen</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C41" t="n">
         <v>0</v>
@@ -16813,7 +16900,7 @@
         <v>0</v>
       </c>
       <c r="G41" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -16822,17 +16909,20 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>93</v>
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
-          <t>Shardul Thakur</t>
+          <t>Tristan Stubbs</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C42" t="n">
         <v>0</v>
@@ -16853,20 +16943,23 @@
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
-          <t>Shubham Dubey</t>
+          <t>Sherfane Rutherford</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="C43" t="n">
         <v>0</v>
@@ -16881,7 +16974,7 @@
         <v>0</v>
       </c>
       <c r="G43" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -16890,17 +16983,20 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
+        <v>93</v>
+      </c>
+      <c r="K43" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
-          <t>Naman Dhir</t>
+          <t>Shardul Thakur</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C44" t="n">
         <v>0</v>
@@ -16918,23 +17014,26 @@
         <v>0</v>
       </c>
       <c r="H44" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
-          <t>Rajat Patidar</t>
+          <t>Shubham Dubey</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C45" t="n">
         <v>0</v>
@@ -16946,10 +17045,10 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -16958,17 +17057,20 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
-          <t>Liam Livingstone</t>
+          <t>Naman Dhir</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C46" t="n">
         <v>0</v>
@@ -16980,29 +17082,32 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>86</v>
+        <v>0</v>
       </c>
       <c r="G46" t="n">
         <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>88</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
       </c>
       <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
-          <t>Shubman Gill</t>
+          <t>Rajat Patidar</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C47" t="n">
         <v>0</v>
@@ -17014,7 +17119,7 @@
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>87</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
@@ -17026,17 +17131,20 @@
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>86</v>
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
-          <t>Nitish Reddy</t>
+          <t>Liam Livingstone</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C48" t="n">
         <v>0</v>
@@ -17048,10 +17156,10 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="G48" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -17060,17 +17168,20 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
-          <t>Faf Du Plessis</t>
+          <t>Shubman Gill</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C49" t="n">
         <v>0</v>
@@ -17091,16 +17202,19 @@
         <v>0</v>
       </c>
       <c r="I49" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="J49" t="n">
+        <v>86</v>
+      </c>
+      <c r="K49" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>Ravi Bishnoi</t>
+          <t>Nitish Reddy</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -17119,26 +17233,29 @@
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
       </c>
       <c r="I50" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
-          <t>Tilak Varma</t>
+          <t>Faf Du Plessis</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="C51" t="n">
         <v>0</v>
@@ -17156,23 +17273,26 @@
         <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="inlineStr">
         <is>
-          <t>Ravindra Jadeja</t>
+          <t>Ravi Bishnoi</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="C52" t="n">
         <v>0</v>
@@ -17190,23 +17310,26 @@
         <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
-          <t>David Miller</t>
+          <t>Tilak Varma</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C53" t="n">
         <v>0</v>
@@ -17224,23 +17347,26 @@
         <v>0</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="I53" t="n">
-        <v>65</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
-          <t>Yash Dayal</t>
+          <t>Ravindra Jadeja</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C54" t="n">
         <v>0</v>
@@ -17252,29 +17378,32 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="G54" t="n">
         <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
       </c>
       <c r="J54" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>Ravichandran Ashwin</t>
+          <t>David Miller</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C55" t="n">
         <v>0</v>
@@ -17292,23 +17421,26 @@
         <v>0</v>
       </c>
       <c r="H55" t="n">
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="J55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="1" t="inlineStr">
         <is>
-          <t>Angkrish Raghuvanshi</t>
+          <t>Yash Dayal</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="C56" t="n">
         <v>0</v>
@@ -17320,7 +17452,7 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="G56" t="n">
         <v>0</v>
@@ -17332,17 +17464,20 @@
         <v>0</v>
       </c>
       <c r="J56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
-          <t>Nathan Ellis</t>
+          <t>Ravichandran Ashwin</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C57" t="n">
         <v>0</v>
@@ -17360,23 +17495,26 @@
         <v>0</v>
       </c>
       <c r="H57" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="I57" t="n">
         <v>0</v>
       </c>
       <c r="J57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
-          <t>Suryakumar Yadav</t>
+          <t>Angkrish Raghuvanshi</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C58" t="n">
         <v>0</v>
@@ -17388,29 +17526,32 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="G58" t="n">
         <v>0</v>
       </c>
       <c r="H58" t="n">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
-          <t>Kagiso Rabada</t>
+          <t>Nathan Ellis</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C59" t="n">
         <v>0</v>
@@ -17428,23 +17569,26 @@
         <v>0</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="I59" t="n">
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>51</v>
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
-          <t>Varun Chakaravarthy</t>
+          <t>Kagiso Rabada</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C60" t="n">
         <v>0</v>
@@ -17456,7 +17600,7 @@
         <v>0</v>
       </c>
       <c r="F60" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="G60" t="n">
         <v>0</v>
@@ -17468,17 +17612,20 @@
         <v>0</v>
       </c>
       <c r="J60" t="n">
+        <v>51</v>
+      </c>
+      <c r="K60" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="1" t="inlineStr">
         <is>
-          <t>Rasikh Dar Salam</t>
+          <t>Varun Chakaravarthy</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C61" t="n">
         <v>0</v>
@@ -17490,7 +17637,7 @@
         <v>0</v>
       </c>
       <c r="F61" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G61" t="n">
         <v>0</v>
@@ -17502,17 +17649,20 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="1" t="inlineStr">
         <is>
-          <t>Suyash Sharma</t>
+          <t>Rasikh Dar Salam</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C62" t="n">
         <v>0</v>
@@ -17524,7 +17674,7 @@
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
@@ -17536,17 +17686,20 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr">
         <is>
-          <t>Marco Jansen</t>
+          <t>Suyash Sharma</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C63" t="n">
         <v>0</v>
@@ -17558,7 +17711,7 @@
         <v>0</v>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="G63" t="n">
         <v>0</v>
@@ -17570,17 +17723,20 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>42</v>
+        <v>0</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr">
         <is>
-          <t>Rinku Singh</t>
+          <t>Marco Jansen</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C64" t="n">
         <v>0</v>
@@ -17592,7 +17748,7 @@
         <v>0</v>
       </c>
       <c r="F64" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G64" t="n">
         <v>0</v>
@@ -17604,17 +17760,20 @@
         <v>0</v>
       </c>
       <c r="J64" t="n">
+        <v>42</v>
+      </c>
+      <c r="K64" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="1" t="inlineStr">
         <is>
-          <t>Mohammed Shami</t>
+          <t>Rinku Singh</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C65" t="n">
         <v>0</v>
@@ -17626,10 +17785,10 @@
         <v>0</v>
       </c>
       <c r="F65" t="n">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="G65" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
@@ -17638,13 +17797,16 @@
         <v>0</v>
       </c>
       <c r="J65" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="1" t="inlineStr">
         <is>
-          <t>Rashid Khan</t>
+          <t>Mohammed Shami</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -17663,7 +17825,7 @@
         <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
@@ -17672,17 +17834,20 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>36</v>
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="1" t="inlineStr">
         <is>
-          <t>Nitish Rana</t>
+          <t>Rashid Khan</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C67" t="n">
         <v>0</v>
@@ -17697,7 +17862,7 @@
         <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
@@ -17706,13 +17871,16 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
+        <v>36</v>
+      </c>
+      <c r="K67" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1" t="inlineStr">
         <is>
-          <t>Aiden Markram</t>
+          <t>Nitish Rana</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -17731,26 +17899,29 @@
         <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="1" t="inlineStr">
         <is>
-          <t>Adam Zampa</t>
+          <t>Aiden Markram</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C69" t="n">
         <v>0</v>
@@ -17765,22 +17936,25 @@
         <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="1" t="inlineStr">
         <is>
-          <t>Marcus Stoinis</t>
+          <t>Adam Zampa</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -17799,7 +17973,7 @@
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
@@ -17808,17 +17982,20 @@
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>34</v>
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr">
         <is>
-          <t>Arshad Khan</t>
+          <t>Marcus Stoinis</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C71" t="n">
         <v>0</v>
@@ -17842,17 +18019,20 @@
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="1" t="inlineStr">
         <is>
-          <t>Shivam Dube</t>
+          <t>Arshad Khan</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C72" t="n">
         <v>0</v>
@@ -17870,23 +18050,26 @@
         <v>0</v>
       </c>
       <c r="H72" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="I72" t="n">
         <v>0</v>
       </c>
       <c r="J72" t="n">
+        <v>33</v>
+      </c>
+      <c r="K72" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="1" t="inlineStr">
         <is>
-          <t>Sandeep Sharma</t>
+          <t>Shivam Dube</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C73" t="n">
         <v>0</v>
@@ -17901,26 +18084,29 @@
         <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H73" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="I73" t="n">
         <v>0</v>
       </c>
       <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="1" t="inlineStr">
         <is>
-          <t>Ryan Rickelton</t>
+          <t>Sandeep Sharma</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C74" t="n">
         <v>0</v>
@@ -17935,26 +18121,29 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H74" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I74" t="n">
         <v>0</v>
       </c>
       <c r="J74" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="1" t="inlineStr">
         <is>
-          <t>Mukesh Kumar</t>
+          <t>Ryan Rickelton</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C75" t="n">
         <v>0</v>
@@ -17972,19 +18161,22 @@
         <v>0</v>
       </c>
       <c r="H75" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I75" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="1" t="inlineStr">
         <is>
-          <t>Shahbaz Ahmed</t>
+          <t>Mukesh Kumar</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -18012,17 +18204,20 @@
         <v>28</v>
       </c>
       <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="1" t="inlineStr">
         <is>
-          <t>Riyan Parag</t>
+          <t>Shahbaz Ahmed</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C77" t="n">
         <v>0</v>
@@ -18037,26 +18232,29 @@
         <v>0</v>
       </c>
       <c r="G77" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H77" t="n">
         <v>0</v>
       </c>
       <c r="I77" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="1" t="inlineStr">
         <is>
-          <t>Yashasvi Jaiswal</t>
+          <t>Riyan Parag</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C78" t="n">
         <v>0</v>
@@ -18071,7 +18269,7 @@
         <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="H78" t="n">
         <v>0</v>
@@ -18080,17 +18278,20 @@
         <v>0</v>
       </c>
       <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr">
         <is>
-          <t>Harshit Rana</t>
+          <t>Yashasvi Jaiswal</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C79" t="n">
         <v>0</v>
@@ -18102,10 +18303,10 @@
         <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="H79" t="n">
         <v>0</v>
@@ -18114,17 +18315,20 @@
         <v>0</v>
       </c>
       <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr">
         <is>
-          <t>Vijaykumar Vyshak</t>
+          <t>Harshit Rana</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C80" t="n">
         <v>0</v>
@@ -18136,7 +18340,7 @@
         <v>0</v>
       </c>
       <c r="F80" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G80" t="n">
         <v>0</v>
@@ -18148,17 +18352,20 @@
         <v>0</v>
       </c>
       <c r="J80" t="n">
-        <v>19</v>
+        <v>0</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="1" t="inlineStr">
         <is>
-          <t>Vaibhav Arora</t>
+          <t>Vijaykumar Vyshak</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C81" t="n">
         <v>0</v>
@@ -18170,7 +18377,7 @@
         <v>0</v>
       </c>
       <c r="F81" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="G81" t="n">
         <v>0</v>
@@ -18182,17 +18389,20 @@
         <v>0</v>
       </c>
       <c r="J81" t="n">
+        <v>19</v>
+      </c>
+      <c r="K81" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="1" t="inlineStr">
         <is>
-          <t>Trent Boult</t>
+          <t>Vaibhav Arora</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C82" t="n">
         <v>0</v>
@@ -18204,25 +18414,28 @@
         <v>0</v>
       </c>
       <c r="F82" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G82" t="n">
         <v>0</v>
       </c>
       <c r="H82" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="I82" t="n">
         <v>0</v>
       </c>
       <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="inlineStr">
         <is>
-          <t>Ayush Badoni</t>
+          <t>Trent Boult</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -18244,23 +18457,26 @@
         <v>0</v>
       </c>
       <c r="H83" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I83" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="1" t="inlineStr">
         <is>
-          <t>Devdutt Padikkal</t>
+          <t>Ayush Badoni</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C84" t="n">
         <v>0</v>
@@ -18272,7 +18488,7 @@
         <v>0</v>
       </c>
       <c r="F84" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G84" t="n">
         <v>0</v>
@@ -18281,20 +18497,23 @@
         <v>0</v>
       </c>
       <c r="I84" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>Satyanarayana Raju</t>
+          <t>Devdutt Padikkal</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C85" t="n">
         <v>0</v>
@@ -18306,29 +18525,32 @@
         <v>0</v>
       </c>
       <c r="F85" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G85" t="n">
         <v>0</v>
       </c>
       <c r="H85" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I85" t="n">
         <v>0</v>
       </c>
       <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="1" t="inlineStr">
         <is>
-          <t>Aniket Verma</t>
+          <t>Satyanarayana Raju</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C86" t="n">
         <v>0</v>
@@ -18343,22 +18565,25 @@
         <v>0</v>
       </c>
       <c r="G86" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H86" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I86" t="n">
         <v>0</v>
       </c>
       <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="1" t="inlineStr">
         <is>
-          <t>Abhinav Manohar</t>
+          <t>Aniket Verma</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -18386,13 +18611,16 @@
         <v>0</v>
       </c>
       <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr">
         <is>
-          <t>MS Dhoni</t>
+          <t>Abhinav Manohar</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -18411,22 +18639,25 @@
         <v>0</v>
       </c>
       <c r="G88" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H88" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I88" t="n">
         <v>0</v>
       </c>
       <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="1" t="inlineStr">
         <is>
-          <t>Rishabh Pant</t>
+          <t>MS Dhoni</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -18448,19 +18679,22 @@
         <v>0</v>
       </c>
       <c r="H89" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I89" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="1" t="inlineStr">
         <is>
-          <t>Prince Yadav</t>
+          <t>Rishabh Pant</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -18488,17 +18722,20 @@
         <v>10</v>
       </c>
       <c r="J90" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="1" t="inlineStr">
         <is>
-          <t>Azmatullah Omarzai</t>
+          <t>Prince Yadav</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C91" t="n">
         <v>0</v>
@@ -18519,16 +18756,19 @@
         <v>0</v>
       </c>
       <c r="I91" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J91" t="n">
-        <v>9</v>
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="1" t="inlineStr">
         <is>
-          <t>Rahul Tewatia</t>
+          <t>Azmatullah Omarzai</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -18557,12 +18797,15 @@
       </c>
       <c r="J92" t="n">
         <v>9</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="1" t="inlineStr">
         <is>
-          <t>Shahrukh Khan</t>
+          <t>Rahul Tewatia</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -18591,16 +18834,19 @@
       </c>
       <c r="J93" t="n">
         <v>9</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="1" t="inlineStr">
         <is>
-          <t>Venkatesh Iyer</t>
+          <t>Shahrukh Khan</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C94" t="n">
         <v>0</v>
@@ -18612,7 +18858,7 @@
         <v>0</v>
       </c>
       <c r="F94" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G94" t="n">
         <v>0</v>
@@ -18624,13 +18870,16 @@
         <v>0</v>
       </c>
       <c r="J94" t="n">
+        <v>9</v>
+      </c>
+      <c r="K94" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="1" t="inlineStr">
         <is>
-          <t>Pat Cummins</t>
+          <t>Venkatesh Iyer</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -18646,10 +18895,10 @@
         <v>0</v>
       </c>
       <c r="F95" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G95" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H95" t="n">
         <v>0</v>
@@ -18658,17 +18907,20 @@
         <v>0</v>
       </c>
       <c r="J95" t="n">
+        <v>0</v>
+      </c>
+      <c r="K95" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="1" t="inlineStr">
         <is>
-          <t>Quinton de Kock</t>
+          <t>Pat Cummins</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C96" t="n">
         <v>0</v>
@@ -18680,10 +18932,10 @@
         <v>0</v>
       </c>
       <c r="F96" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G96" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H96" t="n">
         <v>0</v>
@@ -18692,13 +18944,16 @@
         <v>0</v>
       </c>
       <c r="J96" t="n">
+        <v>0</v>
+      </c>
+      <c r="K96" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="1" t="inlineStr">
         <is>
-          <t>Andre Russell</t>
+          <t>Quinton de Kock</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -18726,13 +18981,16 @@
         <v>0</v>
       </c>
       <c r="J97" t="n">
+        <v>0</v>
+      </c>
+      <c r="K97" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="1" t="inlineStr">
         <is>
-          <t>Sameer Rizvi</t>
+          <t>Andre Russell</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -18748,7 +19006,7 @@
         <v>0</v>
       </c>
       <c r="F98" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G98" t="n">
         <v>0</v>
@@ -18757,16 +19015,19 @@
         <v>0</v>
       </c>
       <c r="I98" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J98" t="n">
+        <v>0</v>
+      </c>
+      <c r="K98" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="1" t="inlineStr">
         <is>
-          <t>Glenn Maxwell</t>
+          <t>Sameer Rizvi</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -18791,20 +19052,23 @@
         <v>0</v>
       </c>
       <c r="I99" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J99" t="n">
-        <v>6</v>
+        <v>0</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="1" t="inlineStr">
         <is>
-          <t>Spencer Johnson</t>
+          <t>Glenn Maxwell</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C100" t="n">
         <v>0</v>
@@ -18816,7 +19080,7 @@
         <v>0</v>
       </c>
       <c r="F100" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G100" t="n">
         <v>0</v>
@@ -18828,17 +19092,20 @@
         <v>0</v>
       </c>
       <c r="J100" t="n">
+        <v>6</v>
+      </c>
+      <c r="K100" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="1" t="inlineStr">
         <is>
-          <t>Rahul Tripathi</t>
+          <t>Spencer Johnson</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C101" t="n">
         <v>0</v>
@@ -18850,29 +19117,32 @@
         <v>0</v>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G101" t="n">
         <v>0</v>
       </c>
       <c r="H101" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I101" t="n">
         <v>0</v>
       </c>
       <c r="J101" t="n">
+        <v>0</v>
+      </c>
+      <c r="K101" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="1" t="inlineStr">
         <is>
-          <t>Jake Fraser-McGurk</t>
+          <t>Rahul Tripathi</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C102" t="n">
         <v>0</v>
@@ -18890,23 +19160,26 @@
         <v>0</v>
       </c>
       <c r="H102" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J102" t="n">
+        <v>0</v>
+      </c>
+      <c r="K102" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="1" t="inlineStr">
         <is>
-          <t>Matheesha Pathirana</t>
+          <t>Jake Fraser-McGurk</t>
         </is>
       </c>
       <c r="B103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C103" t="n">
         <v>0</v>
@@ -18927,16 +19200,19 @@
         <v>0</v>
       </c>
       <c r="I103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J103" t="n">
+        <v>0</v>
+      </c>
+      <c r="K103" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="1" t="inlineStr">
         <is>
-          <t>Gurjapneet Singh</t>
+          <t>Matheesha Pathirana</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -18964,13 +19240,16 @@
         <v>0</v>
       </c>
       <c r="J104" t="n">
+        <v>0</v>
+      </c>
+      <c r="K104" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="1" t="inlineStr">
         <is>
-          <t>Mohammad Siraj</t>
+          <t>Gurjapneet Singh</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -18998,17 +19277,20 @@
         <v>0</v>
       </c>
       <c r="J105" t="n">
+        <v>0</v>
+      </c>
+      <c r="K105" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="1" t="inlineStr">
         <is>
-          <t>Mitchell Santner</t>
+          <t>Mohammad Siraj</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="C106" t="n">
         <v>0</v>
@@ -19026,19 +19308,22 @@
         <v>0</v>
       </c>
       <c r="H106" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I106" t="n">
         <v>0</v>
       </c>
       <c r="J106" t="n">
+        <v>0</v>
+      </c>
+      <c r="K106" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="1" t="inlineStr">
         <is>
-          <t>Yuzvendra Chahal</t>
+          <t>Mitchell Santner</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -19060,23 +19345,26 @@
         <v>0</v>
       </c>
       <c r="H107" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I107" t="n">
         <v>0</v>
       </c>
       <c r="J107" t="n">
-        <v>-2</v>
+        <v>0</v>
+      </c>
+      <c r="K107" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
-          <t>Ramandeep Singh</t>
+          <t>Yuzvendra Chahal</t>
         </is>
       </c>
       <c r="B108" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="C108" t="n">
         <v>0</v>
@@ -19088,7 +19376,7 @@
         <v>0</v>
       </c>
       <c r="F108" t="n">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="G108" t="n">
         <v>0</v>
@@ -19100,17 +19388,20 @@
         <v>0</v>
       </c>
       <c r="J108" t="n">
+        <v>-2</v>
+      </c>
+      <c r="K108" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="1" t="inlineStr">
         <is>
-          <t>Jofra Archer</t>
+          <t>Ramandeep Singh</t>
         </is>
       </c>
       <c r="B109" t="n">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="C109" t="n">
         <v>0</v>
@@ -19122,10 +19413,10 @@
         <v>0</v>
       </c>
       <c r="F109" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="G109" t="n">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="H109" t="n">
         <v>0</v>
@@ -19134,17 +19425,20 @@
         <v>0</v>
       </c>
       <c r="J109" t="n">
+        <v>0</v>
+      </c>
+      <c r="K109" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="1" t="inlineStr">
         <is>
-          <t>Prasidh Krishna</t>
+          <t>Jofra Archer</t>
         </is>
       </c>
       <c r="B110" t="n">
-        <v>-8</v>
+        <v>-7</v>
       </c>
       <c r="C110" t="n">
         <v>0</v>
@@ -19159,7 +19453,7 @@
         <v>0</v>
       </c>
       <c r="G110" t="n">
-        <v>0</v>
+        <v>-7</v>
       </c>
       <c r="H110" t="n">
         <v>0</v>
@@ -19168,7 +19462,10 @@
         <v>0</v>
       </c>
       <c r="J110" t="n">
-        <v>-8</v>
+        <v>0</v>
+      </c>
+      <c r="K110" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -19204,6 +19501,9 @@
       <c r="J111" t="n">
         <v>0</v>
       </c>
+      <c r="K111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="1" t="inlineStr">
@@ -19238,6 +19538,9 @@
       <c r="J112" t="n">
         <v>0</v>
       </c>
+      <c r="K112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="1" t="inlineStr">
@@ -19272,6 +19575,9 @@
       <c r="J113" t="n">
         <v>-13</v>
       </c>
+      <c r="K113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="1" t="inlineStr">
@@ -19306,6 +19612,9 @@
       <c r="J114" t="n">
         <v>0</v>
       </c>
+      <c r="K114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="1" t="inlineStr">
@@ -19340,6 +19649,9 @@
       <c r="J115" t="n">
         <v>0</v>
       </c>
+      <c r="K115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="1" t="inlineStr">
@@ -19372,6 +19684,9 @@
         <v>0</v>
       </c>
       <c r="J116" t="n">
+        <v>0</v>
+      </c>
+      <c r="K116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -23219,11 +23534,7 @@
       <c r="B2" t="n">
         <v>280</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>0</v>
       </c>
@@ -23822,11 +24133,7 @@
       <c r="B3" t="n">
         <v>770</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
@@ -24425,11 +24732,7 @@
       <c r="B4" t="n">
         <v>268</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
@@ -25028,11 +25331,7 @@
       <c r="B5" t="n">
         <v>39</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
@@ -25631,11 +25930,7 @@
       <c r="B6" t="n">
         <v>0</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
@@ -26234,11 +26529,7 @@
       <c r="B7" t="n">
         <v>62</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
@@ -26837,11 +27128,7 @@
       <c r="B8" t="n">
         <v>348</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
@@ -27440,11 +27727,7 @@
       <c r="B9" t="n">
         <v>32</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
@@ -32118,11 +32401,7 @@
       <c r="B2" t="n">
         <v>159</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>0</v>
       </c>
@@ -32721,11 +33000,7 @@
       <c r="B3" t="n">
         <v>189</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
@@ -33324,11 +33599,7 @@
       <c r="B4" t="n">
         <v>180</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
@@ -33927,11 +34198,7 @@
       <c r="B5" t="n">
         <v>349</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
@@ -34530,11 +34797,7 @@
       <c r="B6" t="n">
         <v>119</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
@@ -35133,11 +35396,7 @@
       <c r="B7" t="n">
         <v>272</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
@@ -35736,11 +35995,7 @@
       <c r="B8" t="n">
         <v>107</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
@@ -36339,11 +36594,7 @@
       <c r="B9" t="n">
         <v>305</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>
@@ -40897,11 +41148,7 @@
       <c r="B2" t="n">
         <v>536</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>0</v>
       </c>
@@ -41500,11 +41747,7 @@
       <c r="B3" t="n">
         <v>15</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0</v>
       </c>
@@ -42103,11 +42346,7 @@
       <c r="B4" t="n">
         <v>278</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
         <v>0</v>
       </c>
@@ -42706,11 +42945,7 @@
       <c r="B5" t="n">
         <v>55</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0</v>
       </c>
@@ -43309,11 +43544,7 @@
       <c r="B6" t="n">
         <v>65</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
         <v>0</v>
       </c>
@@ -43912,11 +44143,7 @@
       <c r="B7" t="n">
         <v>350</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
         <v>0</v>
       </c>
@@ -44515,11 +44742,7 @@
       <c r="B8" t="n">
         <v>157</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
         <v>0</v>
       </c>
@@ -45118,11 +45341,7 @@
       <c r="B9" t="n">
         <v>146</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
         <v>0</v>
       </c>

</xml_diff>